<commit_message>
update test plans to remove scanner
</commit_message>
<xml_diff>
--- a/scripts/codemagic-ci/testing/Regression-Test-Plan-Template-Android-PROD.xlsx
+++ b/scripts/codemagic-ci/testing/Regression-Test-Plan-Template-Android-PROD.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27108"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cbryant/UCSD/Dev/Flutter/campusmobile/scripts/codemagic-ci/testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="13_ncr:1_{C36082B3-4413-2A4F-86EE-A9827EA968F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4C664AB-920B-4580-98F6-6A012F50541F}"/>
+  <xr:revisionPtr revIDLastSave="73" documentId="13_ncr:1_{C36082B3-4413-2A4F-86EE-A9827EA968F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BAA3BA1F-F721-43F4-9978-FCC423253834}"/>
   <bookViews>
     <workbookView xWindow="-34740" yWindow="820" windowWidth="38400" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="72">
   <si>
     <t xml:space="preserve">Regression Test Plan - ${APP_VERSION} - ${BUILD_ENV}  </t>
   </si>
@@ -177,30 +177,6 @@
   </si>
   <si>
     <t>Platform Duty Cycle - ESR iPaaS - UCSD Collab (atlassian.net)</t>
-  </si>
-  <si>
-    <t>Native Scanner (not logged in) link navigates to Profile SSO Login</t>
-  </si>
-  <si>
-    <t>Native Scanner (logged in) link launches Scandit Native Scanner</t>
-  </si>
-  <si>
-    <t>Native Scanner Code128 submission successful and verified</t>
-  </si>
-  <si>
-    <t>Native Scanner Code128 submission failed - duplicate barcode</t>
-  </si>
-  <si>
-    <t>Native Scanner Code128 submission failed - invalid barcode</t>
-  </si>
-  <si>
-    <t>Native Scanner 2D submission successful and verified</t>
-  </si>
-  <si>
-    <t>Native Scanner 2D submission failed - duplicate barcode</t>
-  </si>
-  <si>
-    <t>Native Scanner 2D submission failed - invalid barcode</t>
   </si>
   <si>
     <t>MyStudentChart card launches device browser, loads MyStudentChart login site</t>
@@ -593,7 +569,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -689,19 +665,10 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -717,12 +684,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -954,7 +915,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="A1:V977" headerRowCount="0" headerRowDxfId="24" dataDxfId="23" totalsRowDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="A1:V969" headerRowCount="0" headerRowDxfId="24" dataDxfId="23" totalsRowDxfId="22">
   <tableColumns count="22">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Column1" dataDxfId="21"/>
     <tableColumn id="7" xr3:uid="{8D03039E-341F-453C-AC77-00C23E829E8D}" name="Column4" dataDxfId="20"/>
@@ -1189,7 +1150,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:V977"/>
+  <dimension ref="A1:V969"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="96.5703125" style="10" customWidth="1"/>
@@ -1202,7 +1163,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" s="6" customFormat="1" ht="51.75" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="17" t="s">
@@ -1232,7 +1193,7 @@
       <c r="V1" s="5"/>
     </row>
     <row r="2" spans="1:22" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="45" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="19" t="s">
@@ -1263,20 +1224,20 @@
       <c r="V2" s="5"/>
     </row>
     <row r="3" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A3" s="51" t="s">
+      <c r="A3" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="C3" s="40" t="s">
         <v>6</v>
       </c>
       <c r="D3" s="29"/>
       <c r="E3" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="35" t="s">
+      <c r="F3" s="33" t="s">
         <v>8</v>
       </c>
       <c r="G3" s="1"/>
@@ -1300,8 +1261,8 @@
       <c r="A4" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="38"/>
       <c r="D4" s="29"/>
       <c r="E4" s="28" t="s">
         <v>10</v>
@@ -1330,8 +1291,8 @@
       <c r="A5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="40"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
       <c r="D5" s="29"/>
       <c r="E5" s="28" t="s">
         <v>13</v>
@@ -1360,8 +1321,8 @@
       <c r="A6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
+      <c r="B6" s="37"/>
+      <c r="C6" s="37"/>
       <c r="D6" s="1"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
@@ -1384,8 +1345,8 @@
       <c r="A7" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
       <c r="D7" s="1"/>
       <c r="E7" s="22" t="s">
         <v>17</v>
@@ -1412,8 +1373,8 @@
       <c r="A8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="37"/>
       <c r="D8" s="1"/>
       <c r="E8" s="28" t="s">
         <v>19</v>
@@ -1440,8 +1401,8 @@
       <c r="A9" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="40"/>
-      <c r="C9" s="40"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
       <c r="D9" s="1"/>
       <c r="E9" s="28" t="s">
         <v>21</v>
@@ -1468,8 +1429,8 @@
       <c r="A10" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="40"/>
-      <c r="C10" s="40"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
       <c r="D10" s="1"/>
       <c r="E10" s="28" t="s">
         <v>23</v>
@@ -1496,8 +1457,8 @@
       <c r="A11" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="40"/>
-      <c r="C11" s="40"/>
+      <c r="B11" s="37"/>
+      <c r="C11" s="37"/>
       <c r="D11" s="1"/>
       <c r="E11" s="28" t="s">
         <v>25</v>
@@ -1524,8 +1485,8 @@
       <c r="A12" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="40"/>
-      <c r="C12" s="40"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
       <c r="D12" s="1"/>
       <c r="E12" s="28"/>
       <c r="F12" s="10"/>
@@ -1547,11 +1508,11 @@
       <c r="V12" s="1"/>
     </row>
     <row r="13" spans="1:22" ht="28.5">
-      <c r="A13" s="36" t="s">
+      <c r="A13" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="40"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
       <c r="D13" s="1"/>
       <c r="E13" s="22" t="s">
         <v>28</v>
@@ -1578,8 +1539,8 @@
       <c r="A14" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="42"/>
-      <c r="C14" s="42"/>
+      <c r="B14" s="39"/>
+      <c r="C14" s="39"/>
       <c r="D14" s="1"/>
       <c r="E14" s="30" t="s">
         <v>30</v>
@@ -1606,10 +1567,10 @@
       <c r="A15" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="40"/>
-      <c r="C15" s="40"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
       <c r="D15" s="1"/>
-      <c r="E15" s="38" t="s">
+      <c r="E15" s="35" t="s">
         <v>32</v>
       </c>
       <c r="F15" s="10"/>
@@ -1634,10 +1595,10 @@
       <c r="A16" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="40"/>
-      <c r="C16" s="40"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="37"/>
       <c r="D16" s="1"/>
-      <c r="E16" s="39" t="s">
+      <c r="E16" s="36" t="s">
         <v>34</v>
       </c>
       <c r="F16" s="10"/>
@@ -1662,10 +1623,10 @@
       <c r="A17" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B17" s="40"/>
-      <c r="C17" s="40"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
       <c r="D17" s="1"/>
-      <c r="E17" s="38" t="s">
+      <c r="E17" s="35" t="s">
         <v>36</v>
       </c>
       <c r="G17" s="1"/>
@@ -1689,10 +1650,10 @@
       <c r="A18" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="42"/>
-      <c r="C18" s="42"/>
+      <c r="B18" s="39"/>
+      <c r="C18" s="39"/>
       <c r="D18" s="1"/>
-      <c r="E18" s="39" t="s">
+      <c r="E18" s="36" t="s">
         <v>38</v>
       </c>
       <c r="F18" s="1"/>
@@ -1717,10 +1678,10 @@
       <c r="A19" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="40"/>
-      <c r="C19" s="40"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="37"/>
       <c r="D19" s="1"/>
-      <c r="E19" s="38" t="s">
+      <c r="E19" s="35" t="s">
         <v>40</v>
       </c>
       <c r="F19" s="1"/>
@@ -1745,10 +1706,10 @@
       <c r="A20" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B20" s="40"/>
-      <c r="C20" s="40"/>
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
       <c r="D20" s="1"/>
-      <c r="E20" s="39" t="s">
+      <c r="E20" s="36" t="s">
         <v>42</v>
       </c>
       <c r="F20" s="1"/>
@@ -1773,8 +1734,8 @@
       <c r="A21" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="40"/>
-      <c r="C21" s="40"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
       <c r="D21" s="1"/>
       <c r="E21" s="22" t="s">
         <v>44</v>
@@ -1801,13 +1762,13 @@
       <c r="A22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="40"/>
-      <c r="C22" s="40"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
       <c r="D22" s="1"/>
-      <c r="E22" s="38" t="s">
+      <c r="E22" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="F22" s="47"/>
+      <c r="F22" s="42"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
@@ -1829,8 +1790,8 @@
       <c r="A23" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="40"/>
-      <c r="C23" s="40"/>
+      <c r="B23" s="37"/>
+      <c r="C23" s="37"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
@@ -1855,9 +1816,10 @@
       <c r="A24" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="40"/>
-      <c r="C24" s="40"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
       <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
@@ -1880,9 +1842,10 @@
       <c r="A25" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B25" s="40"/>
-      <c r="C25" s="40"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
       <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
@@ -1905,25 +1868,25 @@
       <c r="A26" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="40"/>
-      <c r="C26" s="40"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="33"/>
-      <c r="H26" s="33"/>
-      <c r="I26" s="33"/>
-      <c r="J26" s="33"/>
-      <c r="K26" s="33"/>
-      <c r="L26" s="33"/>
-      <c r="M26" s="33"/>
-      <c r="N26" s="33"/>
-      <c r="O26" s="33"/>
-      <c r="P26" s="33"/>
-      <c r="Q26" s="33"/>
-      <c r="R26" s="33"/>
-      <c r="S26" s="33"/>
-      <c r="T26" s="33"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
+      <c r="R26" s="1"/>
+      <c r="S26" s="1"/>
+      <c r="T26" s="1"/>
       <c r="U26" s="1"/>
       <c r="V26" s="1"/>
     </row>
@@ -1931,64 +1894,64 @@
       <c r="A27" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B27" s="40"/>
-      <c r="C27" s="40"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="34"/>
-      <c r="F27" s="34"/>
-      <c r="G27" s="34"/>
-      <c r="H27" s="34"/>
-      <c r="I27" s="34"/>
-      <c r="J27" s="34"/>
-      <c r="K27" s="34"/>
-      <c r="L27" s="34"/>
-      <c r="M27" s="34"/>
-      <c r="N27" s="34"/>
-      <c r="O27" s="34"/>
-      <c r="P27" s="34"/>
-      <c r="Q27" s="34"/>
-      <c r="R27" s="34"/>
-      <c r="S27" s="34"/>
-      <c r="T27" s="34"/>
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1"/>
+      <c r="R27" s="1"/>
+      <c r="S27" s="1"/>
+      <c r="T27" s="1"/>
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
     </row>
     <row r="28" spans="1:22">
-      <c r="A28" s="36" t="s">
+      <c r="A28" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="43"/>
-      <c r="C28" s="43"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="33"/>
-      <c r="K28" s="33"/>
-      <c r="L28" s="33"/>
-      <c r="M28" s="33"/>
-      <c r="N28" s="33"/>
-      <c r="O28" s="33"/>
-      <c r="P28" s="33"/>
-      <c r="Q28" s="33"/>
-      <c r="R28" s="33"/>
-      <c r="S28" s="33"/>
-      <c r="T28" s="33"/>
+      <c r="B28" s="37"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1"/>
+      <c r="R28" s="1"/>
+      <c r="S28" s="1"/>
+      <c r="T28" s="1"/>
       <c r="U28" s="1"/>
       <c r="V28" s="1"/>
     </row>
     <row r="29" spans="1:22">
-      <c r="A29" s="37" t="s">
+      <c r="A29" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B29" s="44"/>
-      <c r="C29" s="44"/>
-      <c r="D29" s="1"/>
+      <c r="B29" s="37"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="1"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
@@ -2005,12 +1968,13 @@
       <c r="V29" s="1"/>
     </row>
     <row r="30" spans="1:22">
-      <c r="A30" s="36" t="s">
+      <c r="A30" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B30" s="43"/>
-      <c r="C30" s="43"/>
+      <c r="B30" s="37"/>
+      <c r="C30" s="37"/>
       <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
@@ -2033,8 +1997,8 @@
       <c r="A31" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="B31" s="40"/>
-      <c r="C31" s="40"/>
+      <c r="B31" s="37"/>
+      <c r="C31" s="37"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
@@ -2059,8 +2023,8 @@
       <c r="A32" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B32" s="40"/>
-      <c r="C32" s="40"/>
+      <c r="B32" s="37"/>
+      <c r="C32" s="37"/>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
@@ -2082,11 +2046,11 @@
       <c r="V32" s="1"/>
     </row>
     <row r="33" spans="1:22">
-      <c r="A33" s="7" t="s">
+      <c r="A33" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="40"/>
-      <c r="C33" s="40"/>
+      <c r="B33" s="39"/>
+      <c r="C33" s="39"/>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
@@ -2111,8 +2075,8 @@
       <c r="A34" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B34" s="40"/>
-      <c r="C34" s="40"/>
+      <c r="B34" s="37"/>
+      <c r="C34" s="37"/>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
@@ -2137,8 +2101,8 @@
       <c r="A35" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B35" s="40"/>
-      <c r="C35" s="40"/>
+      <c r="B35" s="37"/>
+      <c r="C35" s="37"/>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
@@ -2160,11 +2124,11 @@
       <c r="V35" s="1"/>
     </row>
     <row r="36" spans="1:22">
-      <c r="A36" s="7" t="s">
+      <c r="A36" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B36" s="40"/>
-      <c r="C36" s="40"/>
+      <c r="B36" s="39"/>
+      <c r="C36" s="39"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
@@ -2189,12 +2153,13 @@
       <c r="A37" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B37" s="40"/>
-      <c r="C37" s="40"/>
-      <c r="D37" s="12"/>
+      <c r="B37" s="37"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="1"/>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
@@ -2214,8 +2179,8 @@
       <c r="A38" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B38" s="40"/>
-      <c r="C38" s="40"/>
+      <c r="B38" s="37"/>
+      <c r="C38" s="37"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
       <c r="F38" s="1"/>
@@ -2240,8 +2205,8 @@
       <c r="A39" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B39" s="40"/>
-      <c r="C39" s="40"/>
+      <c r="B39" s="37"/>
+      <c r="C39" s="37"/>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
@@ -2263,11 +2228,11 @@
       <c r="V39" s="1"/>
     </row>
     <row r="40" spans="1:22">
-      <c r="A40" s="7" t="s">
+      <c r="A40" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="B40" s="40"/>
-      <c r="C40" s="40"/>
+      <c r="B40" s="39"/>
+      <c r="C40" s="39"/>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
@@ -2289,11 +2254,11 @@
       <c r="V40" s="1"/>
     </row>
     <row r="41" spans="1:22">
-      <c r="A41" s="8" t="s">
+      <c r="A41" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B41" s="42"/>
-      <c r="C41" s="42"/>
+      <c r="B41" s="37"/>
+      <c r="C41" s="37"/>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
@@ -2318,8 +2283,8 @@
       <c r="A42" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B42" s="40"/>
-      <c r="C42" s="40"/>
+      <c r="B42" s="37"/>
+      <c r="C42" s="37"/>
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
@@ -2344,8 +2309,8 @@
       <c r="A43" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B43" s="40"/>
-      <c r="C43" s="40"/>
+      <c r="B43" s="37"/>
+      <c r="C43" s="37"/>
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
@@ -2367,11 +2332,11 @@
       <c r="V43" s="1"/>
     </row>
     <row r="44" spans="1:22">
-      <c r="A44" s="8" t="s">
+      <c r="A44" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="B44" s="42"/>
-      <c r="C44" s="42"/>
+      <c r="B44" s="37"/>
+      <c r="C44" s="37"/>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
@@ -2393,11 +2358,11 @@
       <c r="V44" s="1"/>
     </row>
     <row r="45" spans="1:22">
-      <c r="A45" s="7" t="s">
+      <c r="A45" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B45" s="40"/>
-      <c r="C45" s="40"/>
+      <c r="B45" s="39"/>
+      <c r="C45" s="39"/>
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
@@ -2419,11 +2384,11 @@
       <c r="V45" s="1"/>
     </row>
     <row r="46" spans="1:22">
-      <c r="A46" s="7" t="s">
+      <c r="A46" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="B46" s="40"/>
-      <c r="C46" s="40"/>
+      <c r="B46" s="37"/>
+      <c r="C46" s="37"/>
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -2444,12 +2409,12 @@
       <c r="U46" s="1"/>
       <c r="V46" s="1"/>
     </row>
-    <row r="47" spans="1:22">
-      <c r="A47" s="7" t="s">
+    <row r="47" spans="1:22" ht="28.5">
+      <c r="A47" s="41" t="s">
         <v>71</v>
       </c>
-      <c r="B47" s="40"/>
-      <c r="C47" s="40"/>
+      <c r="B47" s="13"/>
+      <c r="C47" s="3"/>
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
@@ -2471,11 +2436,9 @@
       <c r="V47" s="1"/>
     </row>
     <row r="48" spans="1:22">
-      <c r="A48" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="B48" s="42"/>
-      <c r="C48" s="42"/>
+      <c r="A48" s="7"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="3"/>
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
       <c r="F48" s="1"/>
@@ -2497,11 +2460,9 @@
       <c r="V48" s="1"/>
     </row>
     <row r="49" spans="1:22">
-      <c r="A49" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="B49" s="40"/>
-      <c r="C49" s="40"/>
+      <c r="A49" s="7"/>
+      <c r="B49" s="13"/>
+      <c r="C49" s="3"/>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
       <c r="F49" s="1"/>
@@ -2523,11 +2484,9 @@
       <c r="V49" s="1"/>
     </row>
     <row r="50" spans="1:22">
-      <c r="A50" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="B50" s="40"/>
-      <c r="C50" s="40"/>
+      <c r="A50" s="7"/>
+      <c r="B50" s="13"/>
+      <c r="C50" s="3"/>
       <c r="D50" s="1"/>
       <c r="E50" s="1"/>
       <c r="F50" s="1"/>
@@ -2549,11 +2508,9 @@
       <c r="V50" s="1"/>
     </row>
     <row r="51" spans="1:22">
-      <c r="A51" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="B51" s="40"/>
-      <c r="C51" s="40"/>
+      <c r="A51" s="7"/>
+      <c r="B51" s="13"/>
+      <c r="C51" s="3"/>
       <c r="D51" s="1"/>
       <c r="E51" s="1"/>
       <c r="F51" s="1"/>
@@ -2575,11 +2532,9 @@
       <c r="V51" s="1"/>
     </row>
     <row r="52" spans="1:22">
-      <c r="A52" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="B52" s="40"/>
-      <c r="C52" s="40"/>
+      <c r="A52" s="7"/>
+      <c r="B52" s="13"/>
+      <c r="C52" s="3"/>
       <c r="D52" s="1"/>
       <c r="E52" s="1"/>
       <c r="F52" s="1"/>
@@ -2601,11 +2556,9 @@
       <c r="V52" s="1"/>
     </row>
     <row r="53" spans="1:22">
-      <c r="A53" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B53" s="42"/>
-      <c r="C53" s="42"/>
+      <c r="A53" s="7"/>
+      <c r="B53" s="13"/>
+      <c r="C53" s="3"/>
       <c r="D53" s="1"/>
       <c r="E53" s="1"/>
       <c r="F53" s="1"/>
@@ -2627,11 +2580,9 @@
       <c r="V53" s="1"/>
     </row>
     <row r="54" spans="1:22">
-      <c r="A54" s="48" t="s">
-        <v>78</v>
-      </c>
-      <c r="B54" s="40"/>
-      <c r="C54" s="40"/>
+      <c r="A54" s="7"/>
+      <c r="B54" s="13"/>
+      <c r="C54" s="3"/>
       <c r="D54" s="1"/>
       <c r="E54" s="1"/>
       <c r="F54" s="1"/>
@@ -2652,10 +2603,8 @@
       <c r="U54" s="1"/>
       <c r="V54" s="1"/>
     </row>
-    <row r="55" spans="1:22" ht="28.5">
-      <c r="A55" s="46" t="s">
-        <v>79</v>
-      </c>
+    <row r="55" spans="1:22">
+      <c r="A55" s="7"/>
       <c r="B55" s="13"/>
       <c r="C55" s="3"/>
       <c r="D55" s="1"/>
@@ -24614,198 +24563,6 @@
       <c r="U969" s="1"/>
       <c r="V969" s="1"/>
     </row>
-    <row r="970" spans="1:22">
-      <c r="A970" s="7"/>
-      <c r="B970" s="13"/>
-      <c r="C970" s="3"/>
-      <c r="D970" s="1"/>
-      <c r="E970" s="1"/>
-      <c r="F970" s="1"/>
-      <c r="G970" s="1"/>
-      <c r="H970" s="1"/>
-      <c r="I970" s="1"/>
-      <c r="J970" s="1"/>
-      <c r="K970" s="1"/>
-      <c r="L970" s="1"/>
-      <c r="M970" s="1"/>
-      <c r="N970" s="1"/>
-      <c r="O970" s="1"/>
-      <c r="P970" s="1"/>
-      <c r="Q970" s="1"/>
-      <c r="R970" s="1"/>
-      <c r="S970" s="1"/>
-      <c r="T970" s="1"/>
-      <c r="U970" s="1"/>
-      <c r="V970" s="1"/>
-    </row>
-    <row r="971" spans="1:22">
-      <c r="A971" s="7"/>
-      <c r="B971" s="13"/>
-      <c r="C971" s="3"/>
-      <c r="D971" s="1"/>
-      <c r="E971" s="1"/>
-      <c r="F971" s="1"/>
-      <c r="G971" s="1"/>
-      <c r="H971" s="1"/>
-      <c r="I971" s="1"/>
-      <c r="J971" s="1"/>
-      <c r="K971" s="1"/>
-      <c r="L971" s="1"/>
-      <c r="M971" s="1"/>
-      <c r="N971" s="1"/>
-      <c r="O971" s="1"/>
-      <c r="P971" s="1"/>
-      <c r="Q971" s="1"/>
-      <c r="R971" s="1"/>
-      <c r="S971" s="1"/>
-      <c r="T971" s="1"/>
-      <c r="U971" s="1"/>
-      <c r="V971" s="1"/>
-    </row>
-    <row r="972" spans="1:22">
-      <c r="A972" s="7"/>
-      <c r="B972" s="13"/>
-      <c r="C972" s="3"/>
-      <c r="D972" s="1"/>
-      <c r="E972" s="1"/>
-      <c r="F972" s="1"/>
-      <c r="G972" s="1"/>
-      <c r="H972" s="1"/>
-      <c r="I972" s="1"/>
-      <c r="J972" s="1"/>
-      <c r="K972" s="1"/>
-      <c r="L972" s="1"/>
-      <c r="M972" s="1"/>
-      <c r="N972" s="1"/>
-      <c r="O972" s="1"/>
-      <c r="P972" s="1"/>
-      <c r="Q972" s="1"/>
-      <c r="R972" s="1"/>
-      <c r="S972" s="1"/>
-      <c r="T972" s="1"/>
-      <c r="U972" s="1"/>
-      <c r="V972" s="1"/>
-    </row>
-    <row r="973" spans="1:22">
-      <c r="A973" s="7"/>
-      <c r="B973" s="13"/>
-      <c r="C973" s="3"/>
-      <c r="D973" s="1"/>
-      <c r="E973" s="1"/>
-      <c r="F973" s="1"/>
-      <c r="G973" s="1"/>
-      <c r="H973" s="1"/>
-      <c r="I973" s="1"/>
-      <c r="J973" s="1"/>
-      <c r="K973" s="1"/>
-      <c r="L973" s="1"/>
-      <c r="M973" s="1"/>
-      <c r="N973" s="1"/>
-      <c r="O973" s="1"/>
-      <c r="P973" s="1"/>
-      <c r="Q973" s="1"/>
-      <c r="R973" s="1"/>
-      <c r="S973" s="1"/>
-      <c r="T973" s="1"/>
-      <c r="U973" s="1"/>
-      <c r="V973" s="1"/>
-    </row>
-    <row r="974" spans="1:22">
-      <c r="A974" s="7"/>
-      <c r="B974" s="13"/>
-      <c r="C974" s="3"/>
-      <c r="D974" s="1"/>
-      <c r="E974" s="1"/>
-      <c r="F974" s="1"/>
-      <c r="G974" s="1"/>
-      <c r="H974" s="1"/>
-      <c r="I974" s="1"/>
-      <c r="J974" s="1"/>
-      <c r="K974" s="1"/>
-      <c r="L974" s="1"/>
-      <c r="M974" s="1"/>
-      <c r="N974" s="1"/>
-      <c r="O974" s="1"/>
-      <c r="P974" s="1"/>
-      <c r="Q974" s="1"/>
-      <c r="R974" s="1"/>
-      <c r="S974" s="1"/>
-      <c r="T974" s="1"/>
-      <c r="U974" s="1"/>
-      <c r="V974" s="1"/>
-    </row>
-    <row r="975" spans="1:22">
-      <c r="A975" s="7"/>
-      <c r="B975" s="13"/>
-      <c r="C975" s="3"/>
-      <c r="D975" s="1"/>
-      <c r="E975" s="1"/>
-      <c r="F975" s="1"/>
-      <c r="G975" s="1"/>
-      <c r="H975" s="1"/>
-      <c r="I975" s="1"/>
-      <c r="J975" s="1"/>
-      <c r="K975" s="1"/>
-      <c r="L975" s="1"/>
-      <c r="M975" s="1"/>
-      <c r="N975" s="1"/>
-      <c r="O975" s="1"/>
-      <c r="P975" s="1"/>
-      <c r="Q975" s="1"/>
-      <c r="R975" s="1"/>
-      <c r="S975" s="1"/>
-      <c r="T975" s="1"/>
-      <c r="U975" s="1"/>
-      <c r="V975" s="1"/>
-    </row>
-    <row r="976" spans="1:22">
-      <c r="A976" s="7"/>
-      <c r="B976" s="13"/>
-      <c r="C976" s="3"/>
-      <c r="D976" s="1"/>
-      <c r="E976" s="1"/>
-      <c r="F976" s="1"/>
-      <c r="G976" s="1"/>
-      <c r="H976" s="1"/>
-      <c r="I976" s="1"/>
-      <c r="J976" s="1"/>
-      <c r="K976" s="1"/>
-      <c r="L976" s="1"/>
-      <c r="M976" s="1"/>
-      <c r="N976" s="1"/>
-      <c r="O976" s="1"/>
-      <c r="P976" s="1"/>
-      <c r="Q976" s="1"/>
-      <c r="R976" s="1"/>
-      <c r="S976" s="1"/>
-      <c r="T976" s="1"/>
-      <c r="U976" s="1"/>
-      <c r="V976" s="1"/>
-    </row>
-    <row r="977" spans="1:22">
-      <c r="A977" s="7"/>
-      <c r="B977" s="13"/>
-      <c r="C977" s="3"/>
-      <c r="D977" s="1"/>
-      <c r="E977" s="1"/>
-      <c r="F977" s="1"/>
-      <c r="G977" s="1"/>
-      <c r="H977" s="1"/>
-      <c r="I977" s="1"/>
-      <c r="J977" s="1"/>
-      <c r="K977" s="1"/>
-      <c r="L977" s="1"/>
-      <c r="M977" s="1"/>
-      <c r="N977" s="1"/>
-      <c r="O977" s="1"/>
-      <c r="P977" s="1"/>
-      <c r="Q977" s="1"/>
-      <c r="R977" s="1"/>
-      <c r="S977" s="1"/>
-      <c r="T977" s="1"/>
-      <c r="U977" s="1"/>
-      <c r="V977" s="1"/>
-    </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
@@ -24826,12 +24583,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -24840,11 +24591,17 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100231ACC10D748F34BAA0C20ABFA72A7EA" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5b60ada5ef74d917189c377d37311689">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a56c8121-053f-455f-842b-cd566811d075" xmlns:ns3="76f06672-c643-4888-a225-c4422b0e89ee" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f62d863a5068cb9de04048c4fc264cf7" ns2:_="" ns3:_="">
-    <xsd:import namespace="a56c8121-053f-455f-842b-cd566811d075"/>
-    <xsd:import namespace="76f06672-c643-4888-a225-c4422b0e89ee"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F5D778AC6A79A84EAA5B25C5A2BFF7B6" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dba055ea2ef6f995fa2b93dd0ece404c">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3cd0eaed-44fe-4f97-8632-c05a782ebbb7" xmlns:ns3="75164c79-2692-43d6-94a7-34b44bf80abd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f036b67ea408c255de0ae726e51a87d7" ns2:_="" ns3:_="">
+    <xsd:import namespace="3cd0eaed-44fe-4f97-8632-c05a782ebbb7"/>
+    <xsd:import namespace="75164c79-2692-43d6-94a7-34b44bf80abd"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -24853,11 +24610,11 @@
               <xsd:all>
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
                 <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
                 <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -24865,7 +24622,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a56c8121-053f-455f-842b-cd566811d075" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="3cd0eaed-44fe-4f97-8632-c05a782ebbb7" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -24878,26 +24635,26 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="10" nillable="true" ma:displayName="Tags" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="11" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="13" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="12" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+    <xsd:element name="MediaServiceSearchProperties" ma:index="14" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
+        <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="76f06672-c643-4888-a225-c4422b0e89ee" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="75164c79-2692-43d6-94a7-34b44bf80abd" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="13" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -24916,7 +24673,7 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="14" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
@@ -25024,13 +24781,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AF01965-4B53-4043-B5ED-A531E4D3A7B2}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F950C44-5D9B-4216-BB47-9736F024226A}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AF01965-4B53-4043-B5ED-A531E4D3A7B2}"/>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9955847E-8391-40AA-9894-0F9AB4282A14}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{77812C01-33E0-4DBA-98E5-AEF18C6A250D}"/>
 </file>
</xml_diff>